<commit_message>
Style content-page blocks and refine importer
Design migration for the content-page template:
- Style the 10 new blocks (columns-cta-band, columns-headline, carousel-hero,
  carousel-cards, carousel-hotspot, accordion-specs, cards-overlay,
  video-poster, quote-large-caps, cards-news) and the standard accordion
- Extend hero-banner (page-title, story and contained heroes) and
  columns-media (light sections) without changing the homepage
- Remove body font-size-adjust, which shrank the headline font ~28%
- Add page-level styles: floating in-page anchor menu, story text column,
  section titles, download/link lists, two-column FAQ sections
- Importer: nested heroes import as hero-banner (contained); FAQ headings
  keep their line breaks; reports refreshed after re-import

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -52,7 +52,7 @@
     <t>content-page</t>
   </si>
   <si>
-    <t>2026-10-18T02:11:50.142Z</t>
+    <t>2026-10-18T06:05:36.170Z</t>
   </si>
   <si>
     <t>Series Configurator - Build Your Own | International®</t>
@@ -70,7 +70,7 @@
     <t>dealer-network</t>
   </si>
   <si>
-    <t>2026-10-18T02:11:57.436Z</t>
+    <t>2026-10-18T06:05:43.963Z</t>
   </si>
   <si>
     <t>Dealer Network | International®</t>
@@ -109,7 +109,7 @@
     <t>industries</t>
   </si>
   <si>
-    <t>2026-10-18T02:15:04.476Z</t>
+    <t>2026-10-18T06:08:52.553Z</t>
   </si>
   <si>
     <t>Industries | International®</t>
@@ -127,7 +127,7 @@
     <t>our-company</t>
   </si>
   <si>
-    <t>2026-10-18T02:17:43.087Z</t>
+    <t>2026-10-18T06:11:21.498Z</t>
   </si>
   <si>
     <t>Our Company | International®</t>
@@ -145,7 +145,7 @@
     <t>parts</t>
   </si>
   <si>
-    <t>2026-10-18T02:31:36.489Z</t>
+    <t>2026-10-18T06:39:29.693Z</t>
   </si>
   <si>
     <t>Parts | International®</t>
@@ -163,7 +163,7 @@
     <t>power-take-off-calculator</t>
   </si>
   <si>
-    <t>2026-10-18T02:32:07.328Z</t>
+    <t>2026-10-18T06:25:18.230Z</t>
   </si>
   <si>
     <t>Power Take-Off Calculator | International®</t>
@@ -181,7 +181,7 @@
     <t>privacy-notice</t>
   </si>
   <si>
-    <t>2026-10-18T02:32:14.307Z</t>
+    <t>2026-10-18T06:39:00.179Z</t>
   </si>
   <si>
     <t>Privacy Notice | International®</t>
@@ -196,7 +196,7 @@
     <t>services</t>
   </si>
   <si>
-    <t>2026-10-18T02:36:12.186Z</t>
+    <t>2026-10-18T06:29:30.769Z</t>
   </si>
   <si>
     <t>Services | International®</t>
@@ -214,7 +214,7 @@
     <t>terms-of-use</t>
   </si>
   <si>
-    <t>2026-10-18T02:41:13.023Z</t>
+    <t>2026-10-18T06:39:07.969Z</t>
   </si>
   <si>
     <t>Terms of Use | International®</t>
@@ -232,7 +232,7 @@
     <t>dealer-network/prestige-certified</t>
   </si>
   <si>
-    <t>2026-10-18T02:12:05.880Z</t>
+    <t>2026-10-18T06:05:51.164Z</t>
   </si>
   <si>
     <t>Prestige Certified | International®</t>
@@ -250,7 +250,7 @@
     <t>dealer-network/recruitment</t>
   </si>
   <si>
-    <t>2026-10-18T02:12:12.530Z</t>
+    <t>2026-10-18T06:05:59.270Z</t>
   </si>
   <si>
     <t>Technician Recruitment | International®</t>
@@ -268,7 +268,7 @@
     <t>fr/our-company</t>
   </si>
   <si>
-    <t>2026-10-18T02:13:18.979Z</t>
+    <t>2026-10-18T06:07:03.046Z</t>
   </si>
   <si>
     <t>https://www.international.com/fr/our-company</t>
@@ -283,7 +283,7 @@
     <t>industries/construction</t>
   </si>
   <si>
-    <t>2026-10-18T02:15:11.807Z</t>
+    <t>2026-10-18T06:09:00.973Z</t>
   </si>
   <si>
     <t>Construction Solutions | International®</t>
@@ -301,7 +301,7 @@
     <t>industries/government-and-municipal</t>
   </si>
   <si>
-    <t>2026-10-18T02:15:41.796Z</t>
+    <t>2026-10-18T06:09:30.169Z</t>
   </si>
   <si>
     <t>Government and Municipal Solutions | International®</t>
@@ -319,7 +319,7 @@
     <t>industries/private-and-general-freight</t>
   </si>
   <si>
-    <t>2026-10-18T02:16:06.331Z</t>
+    <t>2026-10-18T06:09:51.569Z</t>
   </si>
   <si>
     <t>Private and General Freight Solutions | International®</t>
@@ -337,7 +337,7 @@
     <t>industries/specialized-hauling</t>
   </si>
   <si>
-    <t>2026-10-18T02:16:48.182Z</t>
+    <t>2026-10-18T06:10:28.560Z</t>
   </si>
   <si>
     <t>Specialized Hauling | International®</t>
@@ -355,7 +355,7 @@
     <t>industries/utility</t>
   </si>
   <si>
-    <t>2026-10-18T02:17:12.587Z</t>
+    <t>2026-10-18T06:10:50.805Z</t>
   </si>
   <si>
     <t>Utility Solutions | International®</t>
@@ -370,7 +370,7 @@
     <t>legal/shy-settlement</t>
   </si>
   <si>
-    <t>2026-10-18T02:17:20.794Z</t>
+    <t>2026-10-18T06:10:58.583Z</t>
   </si>
   <si>
     <t>Shy Settlement | International®</t>
@@ -385,7 +385,7 @@
     <t>our-company/contact</t>
   </si>
   <si>
-    <t>2026-10-18T02:17:51.187Z</t>
+    <t>2026-10-18T06:11:28.377Z</t>
   </si>
   <si>
     <t>Contact Us | International®</t>
@@ -403,7 +403,7 @@
     <t>our-company/governance</t>
   </si>
   <si>
-    <t>2026-10-18T02:17:59.179Z</t>
+    <t>2026-10-18T06:11:37.128Z</t>
   </si>
   <si>
     <t>Governance | International®</t>
@@ -421,7 +421,7 @@
     <t>our-company/investors</t>
   </si>
   <si>
-    <t>2026-10-18T02:18:08.746Z</t>
+    <t>2026-10-18T06:11:45.964Z</t>
   </si>
   <si>
     <t>Investors | International®</t>
@@ -436,7 +436,7 @@
     <t>our-company/locations</t>
   </si>
   <si>
-    <t>2026-10-18T02:18:16.515Z</t>
+    <t>2026-10-18T06:11:52.994Z</t>
   </si>
   <si>
     <t>Locations | International®</t>
@@ -454,7 +454,7 @@
     <t>our-company/partnerships</t>
   </si>
   <si>
-    <t>2026-10-18T02:18:47.772Z</t>
+    <t>2026-10-18T06:12:25.669Z</t>
   </si>
   <si>
     <t>Partnerships | International®</t>
@@ -472,7 +472,7 @@
     <t>our-company/stories</t>
   </si>
   <si>
-    <t>2026-10-18T02:19:42.125Z</t>
+    <t>2026-10-18T06:13:17.171Z</t>
   </si>
   <si>
     <t>Stories | International®</t>
@@ -490,7 +490,7 @@
     <t>our-company/whistleblower-reporting</t>
   </si>
   <si>
-    <t>2026-10-18T02:31:29.292Z</t>
+    <t>2026-10-18T06:39:23.583Z</t>
   </si>
   <si>
     <t>Whistleblower Reporting | International®</t>
@@ -505,7 +505,7 @@
     <t>parts/global-parts-support</t>
   </si>
   <si>
-    <t>2026-10-18T02:31:43.396Z</t>
+    <t>2026-10-18T06:24:55.377Z</t>
   </si>
   <si>
     <t>Global Parts Support | International®</t>
@@ -523,7 +523,7 @@
     <t>parts/ih-gascap</t>
   </si>
   <si>
-    <t>2026-10-18T02:31:49.742Z</t>
+    <t>2026-10-18T06:25:01.657Z</t>
   </si>
   <si>
     <t>IH Gascap | International®</t>
@@ -541,7 +541,7 @@
     <t>parts/online-ordering</t>
   </si>
   <si>
-    <t>2026-10-18T02:31:56.414Z</t>
+    <t>2026-10-18T06:25:07.304Z</t>
   </si>
   <si>
     <t>Online Parts Ordering | International®</t>
@@ -559,7 +559,7 @@
     <t>products/resources</t>
   </si>
   <si>
-    <t>2026-10-18T02:32:21.782Z</t>
+    <t>2026-10-18T06:25:32.751Z</t>
   </si>
   <si>
     <t>Resources | International®</t>
@@ -577,7 +577,7 @@
     <t>products/trucks</t>
   </si>
   <si>
-    <t>2026-10-18T02:33:34.593Z</t>
+    <t>2026-10-18T06:26:46.373Z</t>
   </si>
   <si>
     <t>Trucks | International®</t>
@@ -595,7 +595,7 @@
     <t>services/financing</t>
   </si>
   <si>
-    <t>2026-10-18T02:36:19.328Z</t>
+    <t>2026-10-18T06:29:37.993Z</t>
   </si>
   <si>
     <t>Financing | International®</t>
@@ -613,7 +613,7 @@
     <t>services/fleet-electrification</t>
   </si>
   <si>
-    <t>2026-10-18T02:37:19.581Z</t>
+    <t>2026-10-18T06:30:39.841Z</t>
   </si>
   <si>
     <t>Fleet Electrification | International®</t>
@@ -631,7 +631,7 @@
     <t>services/fleet-resources</t>
   </si>
   <si>
-    <t>2026-10-18T02:38:06.122Z</t>
+    <t>2026-10-18T06:31:21.764Z</t>
   </si>
   <si>
     <t>Fleet Resources | International®</t>
@@ -646,7 +646,7 @@
     <t>services/global-service-support</t>
   </si>
   <si>
-    <t>2026-10-18T02:38:48.422Z</t>
+    <t>2026-10-18T06:32:05.381Z</t>
   </si>
   <si>
     <t>Global Service Support | International®</t>
@@ -664,7 +664,7 @@
     <t>services/maintenance-services</t>
   </si>
   <si>
-    <t>2026-10-18T02:38:55.320Z</t>
+    <t>2026-10-18T06:32:12.836Z</t>
   </si>
   <si>
     <t>Maintenance Services | International®</t>
@@ -682,7 +682,7 @@
     <t>services/my-international</t>
   </si>
   <si>
-    <t>2026-10-18T02:39:12.303Z</t>
+    <t>2026-10-18T06:32:29.719Z</t>
   </si>
   <si>
     <t>My International™ | International®</t>
@@ -697,7 +697,7 @@
     <t>services/promotions</t>
   </si>
   <si>
-    <t>2026-10-18T02:40:23.506Z</t>
+    <t>2026-10-18T06:33:38.594Z</t>
   </si>
   <si>
     <t>Promotions | International®</t>
@@ -715,7 +715,7 @@
     <t>services/sourcewell</t>
   </si>
   <si>
-    <t>2026-10-18T02:40:37.431Z</t>
+    <t>2026-10-18T06:33:54.474Z</t>
   </si>
   <si>
     <t>Sourcewell Contracts | International®</t>
@@ -733,7 +733,7 @@
     <t>services/uptime-advocate</t>
   </si>
   <si>
-    <t>2026-10-18T02:40:58.985Z</t>
+    <t>2026-10-18T06:34:16.738Z</t>
   </si>
   <si>
     <t>Uptime Advocate | International®</t>
@@ -751,7 +751,7 @@
     <t>services/warranties</t>
   </si>
   <si>
-    <t>2026-10-18T02:41:06.326Z</t>
+    <t>2026-10-18T06:34:23.485Z</t>
   </si>
   <si>
     <t>Warranties | International®</t>
@@ -766,7 +766,7 @@
     <t>dealer-network/recruitment/apply-to-dealership-jobs</t>
   </si>
   <si>
-    <t>2026-10-18T02:12:20.384Z</t>
+    <t>2026-10-18T06:06:06.963Z</t>
   </si>
   <si>
     <t>Dealership Jobs | International®</t>
@@ -784,7 +784,7 @@
     <t>dealer-network/recruitment/become-a-tech</t>
   </si>
   <si>
-    <t>2026-10-18T02:12:28.604Z</t>
+    <t>2026-10-18T06:06:12.611Z</t>
   </si>
   <si>
     <t>Technician Jobs | International®</t>
@@ -802,7 +802,7 @@
     <t>dealer-network/recruitment/influence-winners</t>
   </si>
   <si>
-    <t>2026-10-18T02:12:35.345Z</t>
+    <t>2026-10-18T06:06:19.854Z</t>
   </si>
   <si>
     <t>Technicians of Influence Winners | International®</t>
@@ -820,7 +820,7 @@
     <t>dealer-network/recruitment/internships</t>
   </si>
   <si>
-    <t>2026-10-18T02:12:57.754Z</t>
+    <t>2026-10-18T06:06:40.063Z</t>
   </si>
   <si>
     <t>Internships for Technicians | International®</t>
@@ -838,7 +838,7 @@
     <t>dealer-network/recruitment/service-advisors</t>
   </si>
   <si>
-    <t>2026-10-18T02:13:04.212Z</t>
+    <t>2026-10-18T06:06:46.501Z</t>
   </si>
   <si>
     <t>Service Advisors | International®</t>
@@ -856,7 +856,7 @@
     <t>dealer-network/recruitment/top-team-competition</t>
   </si>
   <si>
-    <t>2026-10-18T02:13:11.282Z</t>
+    <t>2026-10-18T06:06:54.850Z</t>
   </si>
   <si>
     <t>Top Team Technician Competition | International®</t>
@@ -874,7 +874,7 @@
     <t>fr/services/fleet-electrification</t>
   </si>
   <si>
-    <t>2026-10-18T02:14:35.687Z</t>
+    <t>2026-10-18T06:08:19.970Z</t>
   </si>
   <si>
     <t>Électrification des Flottes | International®</t>
@@ -892,7 +892,7 @@
     <t>industries/construction/concrete-mixers</t>
   </si>
   <si>
-    <t>2026-10-18T02:15:18.909Z</t>
+    <t>2026-10-18T06:09:07.145Z</t>
   </si>
   <si>
     <t>Concrete Mixers | International®</t>
@@ -907,7 +907,7 @@
     <t>industries/construction/crane-trucks</t>
   </si>
   <si>
-    <t>2026-10-18T02:15:26.530Z</t>
+    <t>2026-10-18T06:09:15.010Z</t>
   </si>
   <si>
     <t>Crane Trucks | International®</t>
@@ -922,7 +922,7 @@
     <t>industries/construction/dump-trucks</t>
   </si>
   <si>
-    <t>2026-10-18T02:15:32.805Z</t>
+    <t>2026-10-18T06:09:22.414Z</t>
   </si>
   <si>
     <t>Dump Trucks | International®</t>
@@ -937,7 +937,7 @@
     <t>industries/government-and-municipal/fire-and-rescue</t>
   </si>
   <si>
-    <t>2026-10-18T02:15:49.479Z</t>
+    <t>2026-10-18T06:09:35.826Z</t>
   </si>
   <si>
     <t>Fire and Rescue | International®</t>
@@ -952,7 +952,7 @@
     <t>industries/government-and-municipal/snow-plows</t>
   </si>
   <si>
-    <t>2026-10-18T02:15:57.487Z</t>
+    <t>2026-10-18T06:09:43.369Z</t>
   </si>
   <si>
     <t>Snow Plows | International®</t>
@@ -970,7 +970,7 @@
     <t>industries/private-and-general-freight/local-and-regional-delivery</t>
   </si>
   <si>
-    <t>2026-10-18T02:16:15.985Z</t>
+    <t>2026-10-18T06:09:59.708Z</t>
   </si>
   <si>
     <t>Local and Regional Delivery | International®</t>
@@ -988,7 +988,7 @@
     <t>industries/private-and-general-freight/long-haul</t>
   </si>
   <si>
-    <t>2026-10-18T02:16:23.040Z</t>
+    <t>2026-10-18T06:10:05.862Z</t>
   </si>
   <si>
     <t>Long-Haul Trucks | International®</t>
@@ -1003,7 +1003,7 @@
     <t>industries/private-and-general-freight/tankers</t>
   </si>
   <si>
-    <t>2026-10-18T02:16:31.421Z</t>
+    <t>2026-10-18T06:10:13.231Z</t>
   </si>
   <si>
     <t>Tanker Vehicles | International®</t>
@@ -1021,7 +1021,7 @@
     <t>industries/refuse/waste-and-recycling</t>
   </si>
   <si>
-    <t>2026-10-18T02:16:39.308Z</t>
+    <t>2026-10-18T06:10:21.069Z</t>
   </si>
   <si>
     <t>Waste and Recycling Solutions | International®</t>
@@ -1036,7 +1036,7 @@
     <t>industries/specialized-hauling/heavy-haul</t>
   </si>
   <si>
-    <t>2026-10-18T02:16:56.416Z</t>
+    <t>2026-10-18T06:10:36.208Z</t>
   </si>
   <si>
     <t>Heavy Haul | International®</t>
@@ -1051,7 +1051,7 @@
     <t>industries/specialized-hauling/towing-and-recovery</t>
   </si>
   <si>
-    <t>2026-10-18T02:17:03.851Z</t>
+    <t>2026-10-18T06:10:44.023Z</t>
   </si>
   <si>
     <t>Towing and Recovery | International®</t>
@@ -1066,7 +1066,7 @@
     <t>legal/shy-settlement/important-case-documents</t>
   </si>
   <si>
-    <t>2026-10-18T02:17:27.844Z</t>
+    <t>2026-10-18T06:11:05.086Z</t>
   </si>
   <si>
     <t>Important Case Documents | International®</t>
@@ -1081,7 +1081,7 @@
     <t>legal/shy-settlement/shy-settlement-important-dates</t>
   </si>
   <si>
-    <t>2026-10-18T02:17:34.895Z</t>
+    <t>2026-10-18T06:11:13.811Z</t>
   </si>
   <si>
     <t>Shy Settlement Important Dates | International®</t>
@@ -1099,7 +1099,7 @@
     <t>our-company/locations/parts-distribution-centers</t>
   </si>
   <si>
-    <t>2026-10-18T02:18:24.629Z</t>
+    <t>2026-10-18T06:38:46.383Z</t>
   </si>
   <si>
     <t>Parts Distribution Centers | International®</t>
@@ -1114,7 +1114,7 @@
     <t>our-company/locations/production-plants</t>
   </si>
   <si>
-    <t>2026-10-18T02:18:32.979Z</t>
+    <t>2026-10-18T06:12:08.875Z</t>
   </si>
   <si>
     <t>Production Plants | International®</t>
@@ -1132,7 +1132,7 @@
     <t>our-company/locations/proving-grounds</t>
   </si>
   <si>
-    <t>2026-10-18T02:18:41.096Z</t>
+    <t>2026-10-18T06:12:16.796Z</t>
   </si>
   <si>
     <t>Proving Grounds | International®</t>
@@ -1150,7 +1150,7 @@
     <t>our-company/partnerships/loves</t>
   </si>
   <si>
-    <t>2026-10-18T02:18:54.517Z</t>
+    <t>2026-10-18T06:12:32.519Z</t>
   </si>
   <si>
     <t>Love’s and International® Partnership | International®</t>
@@ -1168,7 +1168,7 @@
     <t>our-company/partnerships/supplier-diversity</t>
   </si>
   <si>
-    <t>2026-10-18T02:19:01.724Z</t>
+    <t>2026-10-18T06:38:25.012Z</t>
   </si>
   <si>
     <t>Supplier Diversity | International®</t>
@@ -1186,7 +1186,7 @@
     <t>our-company/people/dei</t>
   </si>
   <si>
-    <t>2026-10-18T02:19:09.886Z</t>
+    <t>2026-10-18T06:12:48.181Z</t>
   </si>
   <si>
     <t>Diversity, Equity And Inclusion | International®</t>
@@ -1204,7 +1204,7 @@
     <t>our-company/people/employee-resource-groups</t>
   </si>
   <si>
-    <t>2026-10-18T02:19:16.580Z</t>
+    <t>2026-10-18T06:12:54.673Z</t>
   </si>
   <si>
     <t>Employee Resource Groups | International®</t>
@@ -1222,7 +1222,7 @@
     <t>our-company/people/leadership</t>
   </si>
   <si>
-    <t>2026-10-18T02:19:24.847Z</t>
+    <t>2026-10-18T06:13:01.706Z</t>
   </si>
   <si>
     <t>Leadership and Executive Management | International®</t>
@@ -1240,7 +1240,7 @@
     <t>our-company/people/retirees</t>
   </si>
   <si>
-    <t>2026-10-18T02:19:33.904Z</t>
+    <t>2026-10-18T06:38:53.174Z</t>
   </si>
   <si>
     <t>Retirees | International®</t>
@@ -1258,7 +1258,7 @@
     <t>products/resources/literature</t>
   </si>
   <si>
-    <t>2026-10-18T02:32:28.461Z</t>
+    <t>2026-10-18T06:25:40.370Z</t>
   </si>
   <si>
     <t>Literature | International®</t>
@@ -1276,7 +1276,7 @@
     <t>products/resources/tem-body-builder</t>
   </si>
   <si>
-    <t>2026-10-18T02:32:41.587Z</t>
+    <t>2026-10-18T06:25:52.886Z</t>
   </si>
   <si>
     <t>TEM Body Builder Resources | International®</t>
@@ -1294,7 +1294,7 @@
     <t>products/trucks/all-electric-refrigerated-truck</t>
   </si>
   <si>
-    <t>2026-10-18T02:33:40.889Z</t>
+    <t>2026-10-18T06:26:54.688Z</t>
   </si>
   <si>
     <t>All Electric Refrigerated Truck | International®</t>
@@ -1312,7 +1312,7 @@
     <t>products/trucks/features</t>
   </si>
   <si>
-    <t>2026-10-18T02:34:09.957Z</t>
+    <t>2026-10-18T06:27:25.524Z</t>
   </si>
   <si>
     <t>Features | International®</t>
@@ -1327,7 +1327,7 @@
     <t>products/trucks/inventory</t>
   </si>
   <si>
-    <t>2026-10-18T02:35:02.652Z</t>
+    <t>2026-10-18T06:28:17.967Z</t>
   </si>
   <si>
     <t>Vehicle Inventory | International®</t>
@@ -1345,7 +1345,7 @@
     <t>products/trucks/legacy-trucks</t>
   </si>
   <si>
-    <t>2026-10-18T02:35:09.055Z</t>
+    <t>2026-10-18T06:28:25.030Z</t>
   </si>
   <si>
     <t>Legacy Models | International®</t>
@@ -1363,7 +1363,7 @@
     <t>services/financing/ev-fleet</t>
   </si>
   <si>
-    <t>2026-10-18T02:36:28.193Z</t>
+    <t>2026-10-18T06:29:45.773Z</t>
   </si>
   <si>
     <t>EV Fleet Financing | International®</t>
@@ -1381,7 +1381,7 @@
     <t>services/financing/financing-canada</t>
   </si>
   <si>
-    <t>2026-10-18T02:36:35.027Z</t>
+    <t>2026-10-18T06:29:53.146Z</t>
   </si>
   <si>
     <t>Financing Canada | International®</t>
@@ -1399,7 +1399,7 @@
     <t>services/financing/leasing</t>
   </si>
   <si>
-    <t>2026-10-18T02:36:42.637Z</t>
+    <t>2026-10-18T06:30:01.370Z</t>
   </si>
   <si>
     <t>Truck and Bus Leasing | International®</t>
@@ -1417,7 +1417,7 @@
     <t>services/financing/loans</t>
   </si>
   <si>
-    <t>2026-10-18T02:36:49.575Z</t>
+    <t>2026-10-18T06:30:10.256Z</t>
   </si>
   <si>
     <t>Commercial Vehicle Loans | International®</t>
@@ -1435,7 +1435,7 @@
     <t>services/financing/municipal-financing</t>
   </si>
   <si>
-    <t>2026-10-18T02:36:55.947Z</t>
+    <t>2026-10-18T06:30:17.071Z</t>
   </si>
   <si>
     <t>Municipal Financing | International®</t>
@@ -1450,7 +1450,7 @@
     <t>services/financing/used-vehicles</t>
   </si>
   <si>
-    <t>2026-10-18T02:37:03.938Z</t>
+    <t>2026-10-18T06:30:24.330Z</t>
   </si>
   <si>
     <t>Used Vehicle Financing Solutions | International®</t>
@@ -1468,7 +1468,7 @@
     <t>services/financing/year-end-cash-in-hand</t>
   </si>
   <si>
-    <t>2026-10-18T02:37:12.807Z</t>
+    <t>2026-10-18T06:30:32.217Z</t>
   </si>
   <si>
     <t>Year End Cash In Hand | International®</t>
@@ -1486,7 +1486,7 @@
     <t>services/fleet-electrification/charging</t>
   </si>
   <si>
-    <t>2026-10-18T02:37:27.586Z</t>
+    <t>2026-10-18T06:38:31.471Z</t>
   </si>
   <si>
     <t>Vehicle Charging | International®</t>
@@ -1504,7 +1504,7 @@
     <t>services/fleet-electrification/consulting</t>
   </si>
   <si>
-    <t>2026-10-18T02:37:34.210Z</t>
+    <t>2026-10-18T06:30:54.351Z</t>
   </si>
   <si>
     <t>Consulting | International®</t>
@@ -1522,7 +1522,7 @@
     <t>services/fleet-electrification/customer-onboarding</t>
   </si>
   <si>
-    <t>2026-10-18T02:37:43.269Z</t>
+    <t>2026-10-18T06:31:01.564Z</t>
   </si>
   <si>
     <t>Customer Onboarding | International®</t>
@@ -1540,7 +1540,7 @@
     <t>services/fleet-electrification/ev-podcast</t>
   </si>
   <si>
-    <t>2026-10-18T02:37:50.900Z</t>
+    <t>2026-10-18T06:31:08.487Z</t>
   </si>
   <si>
     <t>EV Podcast | International®</t>
@@ -1558,7 +1558,7 @@
     <t>services/fleet-electrification/faq</t>
   </si>
   <si>
-    <t>2026-10-18T02:38:00.190Z</t>
+    <t>2026-10-18T06:38:18.310Z</t>
   </si>
   <si>
     <t>FAQ | International®</t>
@@ -1576,7 +1576,7 @@
     <t>services/fleet-resources/emergency-breakdown</t>
   </si>
   <si>
-    <t>2026-10-18T02:38:12.781Z</t>
+    <t>2026-10-18T06:31:29.183Z</t>
   </si>
   <si>
     <t>Emergency Breakdown | International®</t>
@@ -1591,7 +1591,7 @@
     <t>services/fleet-resources/parts-information</t>
   </si>
   <si>
-    <t>2026-10-18T02:38:20.225Z</t>
+    <t>2026-10-18T06:31:37.217Z</t>
   </si>
   <si>
     <t>Parts Information | International®</t>
@@ -1606,7 +1606,7 @@
     <t>services/fleet-resources/parts-return-program</t>
   </si>
   <si>
-    <t>2026-10-18T02:38:27.734Z</t>
+    <t>2026-10-18T06:31:44.794Z</t>
   </si>
   <si>
     <t>Parts Return Program | International®</t>
@@ -1621,7 +1621,7 @@
     <t>services/fleet-resources/service-information</t>
   </si>
   <si>
-    <t>2026-10-18T02:38:34.290Z</t>
+    <t>2026-10-18T06:31:51.903Z</t>
   </si>
   <si>
     <t>Service Information | International®</t>
@@ -1636,7 +1636,7 @@
     <t>services/fleet-resources/technician-education</t>
   </si>
   <si>
-    <t>2026-10-18T02:38:41.836Z</t>
+    <t>2026-10-18T06:31:59.569Z</t>
   </si>
   <si>
     <t>Education Training Program for Technicians | International®</t>
@@ -1654,7 +1654,7 @@
     <t>services/maintenance-services/accelerated-service</t>
   </si>
   <si>
-    <t>2026-10-18T02:39:04.089Z</t>
+    <t>2026-10-18T06:39:43.972Z</t>
   </si>
   <si>
     <t>Accelerated Service | International®</t>
@@ -1672,7 +1672,7 @@
     <t>services/my-international/advanced-remote-diagnostics</t>
   </si>
   <si>
-    <t>2026-10-18T02:39:21.210Z</t>
+    <t>2026-10-18T06:32:36.378Z</t>
   </si>
   <si>
     <t>Advanced Remote Diagnostics | International®</t>
@@ -1690,7 +1690,7 @@
     <t>services/my-international/fuel-analytics</t>
   </si>
   <si>
-    <t>2026-10-18T02:39:28.315Z</t>
+    <t>2026-10-18T06:32:42.345Z</t>
   </si>
   <si>
     <t>Fuel Analytics | International®</t>
@@ -1708,7 +1708,7 @@
     <t>services/my-international/integrations</t>
   </si>
   <si>
-    <t>2026-10-18T02:39:34.917Z</t>
+    <t>2026-10-18T06:39:50.772Z</t>
   </si>
   <si>
     <t>Integrations | International®</t>
@@ -1723,7 +1723,7 @@
     <t>services/my-international/over-the-air-programming</t>
   </si>
   <si>
-    <t>2026-10-18T02:39:41.837Z</t>
+    <t>2026-10-18T06:32:57.138Z</t>
   </si>
   <si>
     <t>Over The Air Programming | International®</t>
@@ -1738,7 +1738,7 @@
     <t>services/my-international/qrcode</t>
   </si>
   <si>
-    <t>2026-10-18T02:39:48.153Z</t>
+    <t>2026-10-18T06:33:04.516Z</t>
   </si>
   <si>
     <t>QR Code | International®</t>
@@ -1756,7 +1756,7 @@
     <t>services/my-international/remote-lock-unlock</t>
   </si>
   <si>
-    <t>2026-10-18T02:39:56.612Z</t>
+    <t>2026-10-18T06:33:10.517Z</t>
   </si>
   <si>
     <t>Remote Lock Unlock | International®</t>
@@ -1774,7 +1774,7 @@
     <t>services/my-international/service-communications</t>
   </si>
   <si>
-    <t>2026-10-18T02:40:04.822Z</t>
+    <t>2026-10-18T06:33:17.434Z</t>
   </si>
   <si>
     <t>Service Communications | International®</t>
@@ -1789,7 +1789,7 @@
     <t>services/my-international/telematics-opt-out</t>
   </si>
   <si>
-    <t>2026-10-18T02:40:11.006Z</t>
+    <t>2026-10-18T06:33:23.709Z</t>
   </si>
   <si>
     <t>Telematics Opt-Out | International®</t>
@@ -1807,7 +1807,7 @@
     <t>services/my-international/terms-of-use-and-privacy-policy</t>
   </si>
   <si>
-    <t>2026-10-18T02:40:17.355Z</t>
+    <t>2026-10-18T06:39:57.954Z</t>
   </si>
   <si>
     <t>Terms of Use and Privacy Policy | International®</t>
@@ -1822,7 +1822,7 @@
     <t>services/promotions/ready-to-roll</t>
   </si>
   <si>
-    <t>2026-10-18T02:40:30.640Z</t>
+    <t>2026-10-18T06:33:47.310Z</t>
   </si>
   <si>
     <t>Earn Up to $1,000 Toward Future Parts &amp; Maintenance | International®</t>
@@ -1840,7 +1840,7 @@
     <t>services/sourcewell/sourcewell-parts</t>
   </si>
   <si>
-    <t>2026-10-18T02:40:43.814Z</t>
+    <t>2026-10-18T06:40:04.935Z</t>
   </si>
   <si>
     <t>Sourcewell Parts | International®</t>
@@ -1858,7 +1858,7 @@
     <t>services/sourcewell/sourcewell-truck</t>
   </si>
   <si>
-    <t>2026-10-18T02:40:51.179Z</t>
+    <t>2026-10-18T06:39:15.878Z</t>
   </si>
   <si>
     <t>Sourcewell Truck | International®</t>
@@ -1876,7 +1876,7 @@
     <t>fr/services/fleet-electrification/charging</t>
   </si>
   <si>
-    <t>2026-10-18T02:14:44.092Z</t>
+    <t>2026-10-18T06:38:39.671Z</t>
   </si>
   <si>
     <t>Recharge | International®</t>
@@ -1891,7 +1891,7 @@
     <t>fr/services/fleet-electrification/consulting</t>
   </si>
   <si>
-    <t>2026-10-18T02:14:50.987Z</t>
+    <t>2026-10-18T06:08:37.693Z</t>
   </si>
   <si>
     <t>Consultation | International®</t>
@@ -1906,7 +1906,7 @@
     <t>fr/services/fleet-electrification/customer-onboarding</t>
   </si>
   <si>
-    <t>2026-10-18T02:14:58.288Z</t>
+    <t>2026-10-18T06:08:43.819Z</t>
   </si>
   <si>
     <t>Intégration des clients | International®</t>
@@ -1921,7 +1921,7 @@
     <t>our-company/stories/2022/2022-carb-emissions-regulations</t>
   </si>
   <si>
-    <t>2026-10-18T02:19:50.407Z</t>
+    <t>2026-10-18T06:13:24.678Z</t>
   </si>
   <si>
     <t>2022 Carb Emissions Regulations | International®</t>
@@ -1936,7 +1936,7 @@
     <t>our-company/stories/2022/2022-truck-trends</t>
   </si>
   <si>
-    <t>2026-10-18T02:19:57.543Z</t>
+    <t>2026-10-18T06:13:32.085Z</t>
   </si>
   <si>
     <t>2022 Truck Trends | International®</t>
@@ -1951,7 +1951,7 @@
     <t>our-company/stories/2022/benefits-of-electric</t>
   </si>
   <si>
-    <t>2026-10-18T02:20:04.755Z</t>
+    <t>2026-10-18T06:13:39.831Z</t>
   </si>
   <si>
     <t>Benefits of Electric | International®</t>
@@ -1969,7 +1969,7 @@
     <t>our-company/stories/2022/charging-ahead</t>
   </si>
   <si>
-    <t>2026-10-18T02:20:12.235Z</t>
+    <t>2026-10-18T06:13:46.544Z</t>
   </si>
   <si>
     <t>Charging Ahead | International®</t>
@@ -1984,7 +1984,7 @@
     <t>our-company/stories/2022/driver-retention</t>
   </si>
   <si>
-    <t>2026-10-18T02:20:18.839Z</t>
+    <t>2026-10-18T06:13:55.255Z</t>
   </si>
   <si>
     <t>Driver Retention | International®</t>
@@ -1999,7 +1999,7 @@
     <t>our-company/stories/2022/emv-walkaround</t>
   </si>
   <si>
-    <t>2026-10-18T02:20:25.173Z</t>
+    <t>2026-10-18T06:14:01.829Z</t>
   </si>
   <si>
     <t>eMV Walkaround | International®</t>
@@ -2014,7 +2014,7 @@
     <t>our-company/stories/2022/lt-series-enhancements</t>
   </si>
   <si>
-    <t>2026-10-18T02:20:31.906Z</t>
+    <t>2026-10-18T06:14:08.671Z</t>
   </si>
   <si>
     <t>LT® Series Enhancements | International®</t>
@@ -2029,7 +2029,7 @@
     <t>our-company/stories/2022/paving-the-way-for-others</t>
   </si>
   <si>
-    <t>2026-10-18T02:20:39.463Z</t>
+    <t>2026-10-18T06:14:15.563Z</t>
   </si>
   <si>
     <t>Paving the Way for Others | International®</t>
@@ -2044,7 +2044,7 @@
     <t>our-company/stories/2022/rose-colored-glasses-breast-cancer-survivor-story</t>
   </si>
   <si>
-    <t>2026-10-18T02:20:47.708Z</t>
+    <t>2026-10-18T06:14:22.227Z</t>
   </si>
   <si>
     <t>Rose-Colored Glasses: My Breast Cancer Survivor Story | International®</t>
@@ -2059,7 +2059,7 @@
     <t>our-company/stories/2022/s13integrated-dual-stage-aftertreatment</t>
   </si>
   <si>
-    <t>2026-10-18T02:20:55.810Z</t>
+    <t>2026-10-18T06:14:29.509Z</t>
   </si>
   <si>
     <t>S13® Integrated Dual Stage Aftertreatment | International®</t>
@@ -2074,7 +2074,7 @@
     <t>our-company/stories/2022/school-busses-will-lead-the-charge-on-electrification</t>
   </si>
   <si>
-    <t>2026-10-18T02:21:05.617Z</t>
+    <t>2026-10-18T06:14:37.854Z</t>
   </si>
   <si>
     <t>School Buses Will Lead The Charge on Electrification | International®</t>
@@ -2089,7 +2089,7 @@
     <t>our-company/stories/2022/the-circle-of-giving-back</t>
   </si>
   <si>
-    <t>2026-10-18T02:21:13.821Z</t>
+    <t>2026-10-18T06:14:46.535Z</t>
   </si>
   <si>
     <t>The Circle of Giving Back | International®</t>
@@ -2104,7 +2104,7 @@
     <t>our-company/stories/2022/truck-maintenance-tips</t>
   </si>
   <si>
-    <t>2026-10-18T02:21:22.248Z</t>
+    <t>2026-10-18T06:14:54.745Z</t>
   </si>
   <si>
     <t>Truck Maintenance Tips | International®</t>
@@ -2119,7 +2119,7 @@
     <t>our-company/stories/2023/2023-truck-trends</t>
   </si>
   <si>
-    <t>2026-10-18T02:21:30.237Z</t>
+    <t>2026-10-18T06:15:02.196Z</t>
   </si>
   <si>
     <t>2023 Truck Trends | International®</t>
@@ -2134,7 +2134,7 @@
     <t>our-company/stories/2023/charging-whitepaper</t>
   </si>
   <si>
-    <t>2026-10-18T02:21:38.641Z</t>
+    <t>2026-10-18T06:15:08.784Z</t>
   </si>
   <si>
     <t>Charging Whitepaper | International®</t>
@@ -2149,7 +2149,7 @@
     <t>our-company/stories/2023/deploying-electric-truck</t>
   </si>
   <si>
-    <t>2026-10-18T02:21:46.259Z</t>
+    <t>2026-10-18T06:15:16.471Z</t>
   </si>
   <si>
     <t>Electric Vehicle Deployment | International®</t>
@@ -2164,7 +2164,7 @@
     <t>our-company/stories/2023/diamond-logic</t>
   </si>
   <si>
-    <t>2026-10-18T02:21:53.385Z</t>
+    <t>2026-10-18T06:15:23.681Z</t>
   </si>
   <si>
     <t>Diamond Logic® | International®</t>
@@ -2179,7 +2179,7 @@
     <t>our-company/stories/2023/electric-vehicle-one-million-miles-driven</t>
   </si>
   <si>
-    <t>2026-10-18T02:22:01.446Z</t>
+    <t>2026-10-18T06:15:29.930Z</t>
   </si>
   <si>
     <t>Electric Truck One Million Miles Driven | International®</t>
@@ -2194,7 +2194,7 @@
     <t>our-company/stories/2023/electric-vehicle-two-million-miles-driven</t>
   </si>
   <si>
-    <t>2026-10-18T02:22:10.816Z</t>
+    <t>2026-10-18T06:15:38.059Z</t>
   </si>
   <si>
     <t>Electric Truck Two Million Miles Driven | International®</t>
@@ -2212,7 +2212,7 @@
     <t>our-company/stories/2023/emv-us-air-conditioning-testimonial</t>
   </si>
   <si>
-    <t>2026-10-18T02:22:20.040Z</t>
+    <t>2026-10-18T06:15:45.804Z</t>
   </si>
   <si>
     <t>eMV US Air Conditioning Testimonial | International®</t>
@@ -2227,7 +2227,7 @@
     <t>our-company/stories/2023/hx-features</t>
   </si>
   <si>
-    <t>2026-10-18T02:22:29.877Z</t>
+    <t>2026-10-18T06:15:53.506Z</t>
   </si>
   <si>
     <t>HX® Features | International®</t>
@@ -2242,7 +2242,7 @@
     <t>our-company/stories/2023/mv-series-safety</t>
   </si>
   <si>
-    <t>2026-10-18T02:22:38.317Z</t>
+    <t>2026-10-18T06:16:02.611Z</t>
   </si>
   <si>
     <t>Safety on the Jobsite and on the Road | International®</t>
@@ -2257,7 +2257,7 @@
     <t>our-company/stories/2023/s13-connected-technologies</t>
   </si>
   <si>
-    <t>2026-10-18T02:22:45.687Z</t>
+    <t>2026-10-18T06:16:10.669Z</t>
   </si>
   <si>
     <t>S13® Connected Technologies | International®</t>
@@ -2272,7 +2272,7 @@
     <t>our-company/stories/2023/supertruck-ii</t>
   </si>
   <si>
-    <t>2026-10-18T02:22:53.093Z</t>
+    <t>2026-10-18T06:16:18.829Z</t>
   </si>
   <si>
     <t>SuperTruck II | International®</t>
@@ -2290,7 +2290,7 @@
     <t>our-company/stories/2023/tackaberry-and-sons</t>
   </si>
   <si>
-    <t>2026-10-18T02:23:02.242Z</t>
+    <t>2026-10-18T06:16:26.235Z</t>
   </si>
   <si>
     <t>Tackaberry and Sons | International®</t>
@@ -2308,7 +2308,7 @@
     <t>our-company/stories/2023/uptime-academy-graduates</t>
   </si>
   <si>
-    <t>2026-10-18T02:23:10.911Z</t>
+    <t>2026-10-18T06:16:34.723Z</t>
   </si>
   <si>
     <t>2022-2023 Uptime Academy Graduates | International®</t>
@@ -2323,7 +2323,7 @@
     <t>our-company/stories/2023/warm-weather-maintenance-tips</t>
   </si>
   <si>
-    <t>2026-10-18T02:23:18.249Z</t>
+    <t>2026-10-18T06:16:42.181Z</t>
   </si>
   <si>
     <t>Warm Weather Maintenance Tips | International®</t>
@@ -2338,7 +2338,7 @@
     <t>our-company/stories/2024/2024-truck-trends</t>
   </si>
   <si>
-    <t>2026-10-18T02:23:26.105Z</t>
+    <t>2026-10-18T06:16:48.930Z</t>
   </si>
   <si>
     <t>2024 Trucking Trends | International®</t>
@@ -2353,7 +2353,7 @@
     <t>our-company/stories/2024/accelerated-service</t>
   </si>
   <si>
-    <t>2026-10-18T02:23:35.187Z</t>
+    <t>2026-10-18T06:16:57.511Z</t>
   </si>
   <si>
     <t>Get Back to Uptime Faster with Accelerated Service | International®</t>
@@ -2368,7 +2368,7 @@
     <t>our-company/stories/2024/an-oems-perspective-on-charging-infrastructure</t>
   </si>
   <si>
-    <t>2026-10-18T02:23:44.767Z</t>
+    <t>2026-10-18T06:17:04.928Z</t>
   </si>
   <si>
     <t>An OEM’s Perspective on Charging Infrastructure for Medium and Heavy-Duty Vehicles—Part 1 | International®</t>
@@ -2386,7 +2386,7 @@
     <t>our-company/stories/2024/autonomous-driving-technology</t>
   </si>
   <si>
-    <t>2026-10-18T02:23:52.529Z</t>
+    <t>2026-10-18T06:17:12.729Z</t>
   </si>
   <si>
     <t>Embracing An Autonomous Future | International®</t>
@@ -2404,7 +2404,7 @@
     <t>our-company/stories/2024/customers-experience-s13-integrated-powertrain</t>
   </si>
   <si>
-    <t>2026-10-18T02:24:01.349Z</t>
+    <t>2026-10-18T06:17:20.239Z</t>
   </si>
   <si>
     <t>Customers Experience S13® Integrated Powertrain | International®</t>
@@ -2419,7 +2419,7 @@
     <t>our-company/stories/2024/driver-safety</t>
   </si>
   <si>
-    <t>2026-10-18T02:24:07.858Z</t>
+    <t>2026-10-18T06:17:26.797Z</t>
   </si>
   <si>
     <t>Safe Driving Tips For Truck Drivers | International®</t>
@@ -2434,7 +2434,7 @@
     <t>our-company/stories/2024/edmonton-parts-distribution-center-success</t>
   </si>
   <si>
-    <t>2026-10-18T02:24:14.571Z</t>
+    <t>2026-10-18T06:17:33.815Z</t>
   </si>
   <si>
     <t>The Story Behind Navistar's Edmonton Parts Distribution Center's Success | International®</t>
@@ -2449,7 +2449,7 @@
     <t>our-company/stories/2024/electric-vehicle-funding</t>
   </si>
   <si>
-    <t>2026-10-18T02:24:23.560Z</t>
+    <t>2026-10-18T06:17:41.722Z</t>
   </si>
   <si>
     <t>How to Navigate Electric Vehicle Funding | International®</t>
@@ -2464,7 +2464,7 @@
     <t>our-company/stories/2024/electric-vehicle-onboarding-part-2</t>
   </si>
   <si>
-    <t>2026-10-18T02:24:40.437Z</t>
+    <t>2026-10-18T06:17:56.939Z</t>
   </si>
   <si>
     <t>Electric Vehicle Onboarding: How Much Power Will Fleets Need for Today, Tomorrow, and Down the Road? | International®</t>
@@ -2479,7 +2479,7 @@
     <t>our-company/stories/2024/electric-vehicle-onboarding</t>
   </si>
   <si>
-    <t>2026-10-18T02:24:32.738Z</t>
+    <t>2026-10-18T06:17:48.622Z</t>
   </si>
   <si>
     <t>Electric Vehicle Onboarding: The Keys to Success for Fleets | International®</t>
@@ -2494,7 +2494,7 @@
     <t>our-company/stories/2024/enhancing-customer-uptime</t>
   </si>
   <si>
-    <t>2026-10-18T02:24:48.785Z</t>
+    <t>2026-10-18T06:18:07.542Z</t>
   </si>
   <si>
     <t>A New Way of Working to Enhance Customer Uptime | International®</t>
@@ -2509,7 +2509,7 @@
     <t>our-company/stories/2024/ev-misconceptions</t>
   </si>
   <si>
-    <t>2026-10-18T02:24:57.685Z</t>
+    <t>2026-10-18T06:18:16.307Z</t>
   </si>
   <si>
     <t>EV misconceptions and facts | International®</t>
@@ -2527,7 +2527,7 @@
     <t>our-company/stories/2024/landscape-trucks</t>
   </si>
   <si>
-    <t>2026-10-18T02:25:04.492Z</t>
+    <t>2026-10-18T06:18:23.738Z</t>
   </si>
   <si>
     <t>The right equipment to grow your business | International®</t>
@@ -2542,7 +2542,7 @@
     <t>our-company/stories/2024/leveraging-history-to-support-customer-needs</t>
   </si>
   <si>
-    <t>2026-10-18T02:25:12.471Z</t>
+    <t>2026-10-18T06:18:31.608Z</t>
   </si>
   <si>
     <t>Navistar Financial Leverages History to Support Everchanging Customer Needs | International®</t>
@@ -2557,7 +2557,7 @@
     <t>our-company/stories/2024/national-school-bus-safety-week</t>
   </si>
   <si>
-    <t>2026-10-18T02:25:18.996Z</t>
+    <t>2026-10-18T06:18:38.953Z</t>
   </si>
   <si>
     <t>National School Bus Safety Week | International®</t>
@@ -2575,7 +2575,7 @@
     <t>our-company/stories/2024/real-world-testing-the-international-s13-integrated-powertrain</t>
   </si>
   <si>
-    <t>2026-10-18T02:25:26.063Z</t>
+    <t>2026-10-18T06:18:47.294Z</t>
   </si>
   <si>
     <t>Real World Testing the International® S13® Integrated Powertrain | International®</t>
@@ -2593,7 +2593,7 @@
     <t>our-company/stories/2024/s13-interview</t>
   </si>
   <si>
-    <t>2026-10-18T02:25:34.228Z</t>
+    <t>2026-10-18T06:18:54.071Z</t>
   </si>
   <si>
     <t>An Interview With S13® Integrated Chief Engineer | International®</t>
@@ -2608,7 +2608,7 @@
     <t>our-company/stories/2024/sustainable-solutions-report</t>
   </si>
   <si>
-    <t>2026-10-18T02:25:41.391Z</t>
+    <t>2026-10-18T06:19:01.300Z</t>
   </si>
   <si>
     <t>International® Sustainable Solutions Special Report | International®</t>
@@ -2623,7 +2623,7 @@
     <t>our-company/stories/2024/the-diesel-to-electric-transition</t>
   </si>
   <si>
-    <t>2026-10-18T02:25:48.304Z</t>
+    <t>2026-10-18T06:19:10.159Z</t>
   </si>
   <si>
     <t>The Diesel to Electric Transition: International® Truck Helps Fleets Prepare | International®</t>
@@ -2638,7 +2638,7 @@
     <t>our-company/stories/2024/tmc-annual-meeting</t>
   </si>
   <si>
-    <t>2026-10-18T02:25:55.857Z</t>
+    <t>2026-10-18T06:19:17.685Z</t>
   </si>
   <si>
     <t>TMC Annual Meeting | International®</t>
@@ -2653,7 +2653,7 @@
     <t>our-company/stories/2024/understanding-fleet-electrification-needs</t>
   </si>
   <si>
-    <t>2026-10-18T02:26:04.213Z</t>
+    <t>2026-10-18T06:19:26.824Z</t>
   </si>
   <si>
     <t>Consulting: Understanding Fleet Electrification Needs | International®</t>
@@ -2671,7 +2671,7 @@
     <t>our-company/stories/2024/world-of-concrete</t>
   </si>
   <si>
-    <t>2026-10-18T02:26:11.241Z</t>
+    <t>2026-10-18T06:19:34.911Z</t>
   </si>
   <si>
     <t>Building Relationships, Cementing Partnerships | International®</t>
@@ -2686,7 +2686,7 @@
     <t>our-company/stories/2024/year-round-maintenance-plan</t>
   </si>
   <si>
-    <t>2026-10-18T02:26:18.658Z</t>
+    <t>2026-10-18T06:19:42.772Z</t>
   </si>
   <si>
     <t>See What Needs To Be In Your Fleet’s Year-Round Maintenance Plan | International®</t>
@@ -2701,7 +2701,7 @@
     <t>our-company/stories/2025/a-finance-partner-that-understands-the-truck-business</t>
   </si>
   <si>
-    <t>2026-10-18T02:26:28.210Z</t>
+    <t>2026-10-18T06:19:50.972Z</t>
   </si>
   <si>
     <t>A finance partner that understands the truck business | International®</t>
@@ -2716,7 +2716,7 @@
     <t>our-company/stories/2025/act-expo-main-stage-panel</t>
   </si>
   <si>
-    <t>2026-10-18T02:26:35.169Z</t>
+    <t>2026-10-18T06:19:59.594Z</t>
   </si>
   <si>
     <t>How software-defined vehicles offer new possibilities | International®</t>
@@ -2731,7 +2731,7 @@
     <t>our-company/stories/2025/building-sustainable-mobility-through-digitalization</t>
   </si>
   <si>
-    <t>2026-10-18T02:26:42.194Z</t>
+    <t>2026-10-18T06:20:07.971Z</t>
   </si>
   <si>
     <t>Building sustainable mobility through digitalization | International®</t>
@@ -2749,7 +2749,7 @@
     <t>our-company/stories/2025/docuseries</t>
   </si>
   <si>
-    <t>2026-10-18T02:26:48.554Z</t>
+    <t>2026-10-18T06:20:15.177Z</t>
   </si>
   <si>
     <t>Documenting the extraordinary lengths drivers go | International®</t>
@@ -2767,7 +2767,7 @@
     <t>our-company/stories/2025/everything-you-need-to-know-about-adding-bev-trucks-to-your-fleet</t>
   </si>
   <si>
-    <t>2026-10-18T02:26:56.958Z</t>
+    <t>2026-10-18T06:20:22.793Z</t>
   </si>
   <si>
     <t>Everything You Need to Know About Adding BEV Trucks to Your Fleet | International®</t>
@@ -2782,7 +2782,7 @@
     <t>our-company/stories/2025/fleet-financial-strategies-for-a-volatile-market</t>
   </si>
   <si>
-    <t>2026-10-18T02:27:03.660Z</t>
+    <t>2026-10-18T06:20:30.150Z</t>
   </si>
   <si>
     <t>Fleet financial strategies for a volatile market | International®</t>
@@ -2797,7 +2797,7 @@
     <t>our-company/stories/2025/hv-series-puts-in-the-work</t>
   </si>
   <si>
-    <t>2026-10-18T02:27:12.958Z</t>
+    <t>2026-10-18T06:20:37.022Z</t>
   </si>
   <si>
     <t>New HV Series puts in the work for hardworking fleets | International®</t>
@@ -2812,7 +2812,7 @@
     <t>our-company/stories/2025/modernizing-an-american-legacy</t>
   </si>
   <si>
-    <t>2026-10-18T02:27:20.495Z</t>
+    <t>2026-10-18T06:20:43.306Z</t>
   </si>
   <si>
     <t>Modernizing an American legacy | International®</t>
@@ -2827,7 +2827,7 @@
     <t>our-company/stories/2025/mv-series-ready-for-any-job</t>
   </si>
   <si>
-    <t>2026-10-18T02:27:29.183Z</t>
+    <t>2026-10-18T06:20:50.841Z</t>
   </si>
   <si>
     <t>MV Series: Ready for any job | International®</t>
@@ -2842,7 +2842,7 @@
     <t>our-company/stories/2025/prairie-farms-fleet</t>
   </si>
   <si>
-    <t>2026-10-18T02:27:36.514Z</t>
+    <t>2026-10-18T06:20:57.125Z</t>
   </si>
   <si>
     <t>Prairie Farms fleet | International®</t>
@@ -2857,7 +2857,7 @@
     <t>our-company/stories/2025/q4-financing-a-new-truck</t>
   </si>
   <si>
-    <t>2026-10-18T02:27:44.231Z</t>
+    <t>2026-10-18T06:21:04.344Z</t>
   </si>
   <si>
     <t>Why is Q4 the smartest time to finance a new truck? | International®</t>
@@ -2872,7 +2872,7 @@
     <t>our-company/stories/2025/s13-integrated-powertrain-for-concrete-mixers</t>
   </si>
   <si>
-    <t>2026-10-18T02:27:53.024Z</t>
+    <t>2026-10-18T06:21:11.065Z</t>
   </si>
   <si>
     <t>S13 Integrated Powertrain: A game-changer for concrete mixers | International®</t>
@@ -2890,7 +2890,7 @@
     <t>our-company/stories/2025/s13-solutions-deliver-for-menzel-enterprises</t>
   </si>
   <si>
-    <t>2026-10-18T02:28:00.966Z</t>
+    <t>2026-10-18T06:21:18.052Z</t>
   </si>
   <si>
     <t>S13 Integrated Powertrain solutions deliver for Menzel Enterprises | International®</t>
@@ -2905,7 +2905,7 @@
     <t>our-company/stories/2025/scott-miller-testimonial</t>
   </si>
   <si>
-    <t>2026-10-18T02:28:11.289Z</t>
+    <t>2026-10-18T06:21:24.847Z</t>
   </si>
   <si>
     <t>Scott Miller Testimonial | International®</t>
@@ -2920,7 +2920,7 @@
     <t>our-company/stories/2025/the-s13-integrated-powertrain-powers-ready-mix-success</t>
   </si>
   <si>
-    <t>2026-10-18T02:28:19.768Z</t>
+    <t>2026-10-18T06:21:31.187Z</t>
   </si>
   <si>
     <t>The S13 Integrated Powertrain powers ready mix success | International®</t>
@@ -2935,7 +2935,7 @@
     <t>our-company/stories/2025/tulsa-bus-plant-250000-unit-milestone</t>
   </si>
   <si>
-    <t>2026-10-18T02:28:27.303Z</t>
+    <t>2026-10-18T06:21:39.125Z</t>
   </si>
   <si>
     <t>Tulsa Bus Plant's 250,000-unit milestone | International®</t>
@@ -2950,7 +2950,7 @@
     <t>our-company/stories/2025/us-air-conditioning</t>
   </si>
   <si>
-    <t>2026-10-18T02:28:36.107Z</t>
+    <t>2026-10-18T06:21:47.372Z</t>
   </si>
   <si>
     <t>U.S. Air Conditioning | International®</t>
@@ -2965,7 +2965,7 @@
     <t>our-company/stories/2026/250-years-of-america</t>
   </si>
   <si>
-    <t>2026-10-18T02:28:43.076Z</t>
+    <t>2026-10-18T06:21:55.978Z</t>
   </si>
   <si>
     <t>250 years of America | International®</t>
@@ -2983,7 +2983,7 @@
     <t>our-company/stories/2026/a-new-approach-to-service-contracts</t>
   </si>
   <si>
-    <t>2026-10-18T02:28:51.558Z</t>
+    <t>2026-10-18T06:22:02.933Z</t>
   </si>
   <si>
     <t>A new approach to service contracts | International®</t>
@@ -2998,7 +2998,7 @@
     <t>our-company/stories/2026/buying-your-first-international-truck</t>
   </si>
   <si>
-    <t>2026-10-18T02:28:59.347Z</t>
+    <t>2026-10-18T06:22:11.000Z</t>
   </si>
   <si>
     <t>Buying your first International truck | International®</t>
@@ -3013,7 +3013,7 @@
     <t>our-company/stories/2026/director-of-powertrain-engineering-named-2025-sae-international-fellow</t>
   </si>
   <si>
-    <t>2026-10-18T02:29:06.953Z</t>
+    <t>2026-10-18T06:22:19.451Z</t>
   </si>
   <si>
     <t>Director of powertrain engineering named 2025 SAE International Fellow | International®</t>
@@ -3028,7 +3028,7 @@
     <t>our-company/stories/2026/how-international-financial-delivers-financing-solutions</t>
   </si>
   <si>
-    <t>2026-10-18T02:29:14.806Z</t>
+    <t>2026-10-18T06:22:26.669Z</t>
   </si>
   <si>
     <t>How International® Financial delivers financing solutions | International®</t>
@@ -3043,7 +3043,7 @@
     <t>our-company/stories/2026/how-my-international-redefines-the-customer-ownership-experience</t>
   </si>
   <si>
-    <t>2026-10-18T02:29:21.407Z</t>
+    <t>2026-10-18T06:22:33.943Z</t>
   </si>
   <si>
     <t>How My International redefines the customer ownership experience | International®</t>
@@ -3058,7 +3058,7 @@
     <t>our-company/stories/2026/how-proactive-maintenance-can-boost-your-uptime</t>
   </si>
   <si>
-    <t>2026-10-18T02:29:27.828Z</t>
+    <t>2026-10-18T06:22:41.573Z</t>
   </si>
   <si>
     <t>How proactive maintenance can boost your uptime | International®</t>
@@ -3073,7 +3073,7 @@
     <t>our-company/stories/2026/international-celebrates-5-years-of-social-impact</t>
   </si>
   <si>
-    <t>2026-10-18T02:29:34.565Z</t>
+    <t>2026-10-18T06:22:48.845Z</t>
   </si>
   <si>
     <t>International celebrates 5 years of Social Impact | International®</t>
@@ -3088,7 +3088,7 @@
     <t>our-company/stories/2026/international-financial-practical-guide</t>
   </si>
   <si>
-    <t>2026-10-18T02:29:41.849Z</t>
+    <t>2026-10-18T06:22:55.664Z</t>
   </si>
   <si>
     <t>International Financial Practical Guide | International®</t>
@@ -3103,7 +3103,7 @@
     <t>our-company/stories/2026/international-named-one-of-the-most-trustworthy-companies</t>
   </si>
   <si>
-    <t>2026-10-18T02:29:50.212Z</t>
+    <t>2026-10-18T06:23:03.404Z</t>
   </si>
   <si>
     <t>International named one of the Most Trustworthy Companies | International®</t>
@@ -3118,7 +3118,7 @@
     <t>our-company/stories/2026/plan-smarter-save-more-with-financing-built-for-your-fleet</t>
   </si>
   <si>
-    <t>2026-10-18T02:29:57.041Z</t>
+    <t>2026-10-18T06:23:10.738Z</t>
   </si>
   <si>
     <t>Plan Smarter: Save more with financing built for your fleet | International®</t>
@@ -3133,7 +3133,7 @@
     <t>our-company/stories/2026/pods-moving-and-storage</t>
   </si>
   <si>
-    <t>2026-10-18T02:30:04.707Z</t>
+    <t>2026-10-18T06:23:19.437Z</t>
   </si>
   <si>
     <t>Reliability is everything for PODS Moving and Storage fleet | International®</t>
@@ -3148,7 +3148,7 @@
     <t>our-company/stories/2026/support-that-goes-beyond-the-sale</t>
   </si>
   <si>
-    <t>2026-10-18T02:30:12.288Z</t>
+    <t>2026-10-18T06:23:28.558Z</t>
   </si>
   <si>
     <t>Support that goes beyond the sale | International®</t>
@@ -3163,7 +3163,7 @@
     <t>our-company/stories/2026/t14-transmission-built-for-the-jobsite</t>
   </si>
   <si>
-    <t>2026-10-18T02:30:21.389Z</t>
+    <t>2026-10-18T06:23:35.178Z</t>
   </si>
   <si>
     <t>T14 Transmission: Built for the jobsite | International®</t>
@@ -3181,7 +3181,7 @@
     <t>our-company/stories/2026/testing-for-improved-truck-fuel-efficiency</t>
   </si>
   <si>
-    <t>2026-10-18T02:30:27.652Z</t>
+    <t>2026-10-18T06:23:42.190Z</t>
   </si>
   <si>
     <t>Testing for improved truck fuel efficiency | International®</t>
@@ -3196,7 +3196,7 @@
     <t>our-company/stories/2026/truck-driver-appreciation</t>
   </si>
   <si>
-    <t>2026-10-18T02:30:35.384Z</t>
+    <t>2026-10-18T06:23:48.353Z</t>
   </si>
   <si>
     <t>Meet the people who call the LT® Series truck home | International®</t>
@@ -3211,7 +3211,7 @@
     <t>our-company/stories/2026/why-international-vocational-trucks-rule-the-jobsite</t>
   </si>
   <si>
-    <t>2026-10-18T02:30:42.711Z</t>
+    <t>2026-10-18T06:23:56.211Z</t>
   </si>
   <si>
     <t>Why International vocational trucks rule the jobsite | International®</t>
@@ -3229,7 +3229,7 @@
     <t>our-company/vision-and-strategy/culture-and-leadership/shared-values</t>
   </si>
   <si>
-    <t>2026-10-18T02:30:49.247Z</t>
+    <t>2026-10-18T06:24:03.769Z</t>
   </si>
   <si>
     <t>Shared Values | International®</t>
@@ -3247,7 +3247,7 @@
     <t>our-company/vision-and-strategy/foundations-for-future/digitalization</t>
   </si>
   <si>
-    <t>2026-10-18T02:30:57.701Z</t>
+    <t>2026-10-18T06:24:11.074Z</t>
   </si>
   <si>
     <t>Digitalization | International®</t>
@@ -3265,7 +3265,7 @@
     <t>our-company/vision-and-strategy/foundations-for-future/electrification</t>
   </si>
   <si>
-    <t>2026-10-18T02:31:05.662Z</t>
+    <t>2026-10-18T06:24:19.480Z</t>
   </si>
   <si>
     <t>Electrification | International®</t>
@@ -3283,7 +3283,7 @@
     <t>our-company/vision-and-strategy/sustainability/environmental-impact</t>
   </si>
   <si>
-    <t>2026-10-18T02:31:15.130Z</t>
+    <t>2026-10-18T06:24:27.169Z</t>
   </si>
   <si>
     <t>Environmental Impact | International®</t>
@@ -3301,7 +3301,7 @@
     <t>our-company/vision-and-strategy/sustainability/social-impact</t>
   </si>
   <si>
-    <t>2026-10-18T02:31:23.009Z</t>
+    <t>2026-10-18T06:39:36.471Z</t>
   </si>
   <si>
     <t>Social Impact | International®</t>
@@ -3319,7 +3319,7 @@
     <t>products/resources/operator-guides-and-training/bev-training-material</t>
   </si>
   <si>
-    <t>2026-10-18T02:32:34.962Z</t>
+    <t>2026-10-18T06:25:46.764Z</t>
   </si>
   <si>
     <t>BEV Training Material | International®</t>
@@ -3334,7 +3334,7 @@
     <t>products/resources/tem-body-builder/body-resources</t>
   </si>
   <si>
-    <t>2026-10-18T02:32:48.204Z</t>
+    <t>2026-10-18T06:25:59.785Z</t>
   </si>
   <si>
     <t>Body Builder Resources | International®</t>
@@ -3352,7 +3352,7 @@
     <t>products/resources/tem-body-builder/cad-data</t>
   </si>
   <si>
-    <t>2026-10-18T02:32:56.707Z</t>
+    <t>2026-10-18T06:26:09.373Z</t>
   </si>
   <si>
     <t>CAD Data Resources | International®</t>
@@ -3370,7 +3370,7 @@
     <t>products/resources/tem-body-builder/engine-resources</t>
   </si>
   <si>
-    <t>2026-10-18T02:33:05.480Z</t>
+    <t>2026-10-18T06:26:17.003Z</t>
   </si>
   <si>
     <t>Engine Resources | International®</t>
@@ -3385,7 +3385,7 @@
     <t>products/resources/tem-body-builder/t14-transmission-resources</t>
   </si>
   <si>
-    <t>2026-10-18T02:33:13.426Z</t>
+    <t>2026-10-18T06:26:24.199Z</t>
   </si>
   <si>
     <t>Transmission Media | International®</t>
@@ -3400,7 +3400,7 @@
     <t>products/resources/tem-body-builder/tips-and-training</t>
   </si>
   <si>
-    <t>2026-10-18T02:33:20.186Z</t>
+    <t>2026-10-18T06:26:31.592Z</t>
   </si>
   <si>
     <t>Tips and Training | International®</t>
@@ -3415,7 +3415,7 @@
     <t>products/resources/tem-body-builder/tools-and-software</t>
   </si>
   <si>
-    <t>2026-10-18T02:33:28.106Z</t>
+    <t>2026-10-18T06:26:39.433Z</t>
   </si>
   <si>
     <t>Tools And Software | International®</t>
@@ -3433,7 +3433,7 @@
     <t>products/trucks/classes/heavy</t>
   </si>
   <si>
-    <t>2026-10-18T02:33:47.026Z</t>
+    <t>2026-10-18T06:27:03.034Z</t>
   </si>
   <si>
     <t>Heavy-Duty Trucks | International®</t>
@@ -3451,7 +3451,7 @@
     <t>products/trucks/classes/medium</t>
   </si>
   <si>
-    <t>2026-10-18T02:33:55.622Z</t>
+    <t>2026-10-18T06:27:10.422Z</t>
   </si>
   <si>
     <t>Medium-Duty Trucks | International®</t>
@@ -3466,7 +3466,7 @@
     <t>products/trucks/classes/severe</t>
   </si>
   <si>
-    <t>2026-10-18T02:34:02.831Z</t>
+    <t>2026-10-18T06:27:17.181Z</t>
   </si>
   <si>
     <t>Severe-Duty Trucks | International®</t>
@@ -3484,7 +3484,7 @@
     <t>products/trucks/features/diamond-logic</t>
   </si>
   <si>
-    <t>2026-10-18T02:34:18.393Z</t>
+    <t>2026-10-18T06:27:33.685Z</t>
   </si>
   <si>
     <t>https://www.international.com/products/trucks/features/diamond-logic</t>
@@ -3499,7 +3499,7 @@
     <t>products/trucks/features/engines-and-powertrains</t>
   </si>
   <si>
-    <t>2026-10-18T02:34:24.944Z</t>
+    <t>2026-10-18T06:27:40.451Z</t>
   </si>
   <si>
     <t>Engines and Powertrains | International®</t>
@@ -3517,7 +3517,7 @@
     <t>products/trucks/legacy-trucks/proven-trucks</t>
   </si>
   <si>
-    <t>2026-10-18T02:35:16.274Z</t>
+    <t>2026-10-18T06:28:32.438Z</t>
   </si>
   <si>
     <t>Proven Trucks | International®</t>
@@ -3535,7 +3535,7 @@
     <t>products/trucks/series/cv</t>
   </si>
   <si>
-    <t>2026-10-18T02:35:24.659Z</t>
+    <t>2026-10-18T06:28:40.622Z</t>
   </si>
   <si>
     <t>CV™ Series | International®</t>
@@ -3553,7 +3553,7 @@
     <t>products/trucks/series/electric-mv</t>
   </si>
   <si>
-    <t>2026-10-18T02:35:33.324Z</t>
+    <t>2026-10-18T06:28:49.178Z</t>
   </si>
   <si>
     <t>eMV™ Series | International®</t>
@@ -3571,7 +3571,7 @@
     <t>products/trucks/series/hv</t>
   </si>
   <si>
-    <t>2026-10-18T02:35:41.127Z</t>
+    <t>2026-10-18T06:28:58.888Z</t>
   </si>
   <si>
     <t>HV™ Series | International®</t>
@@ -3589,7 +3589,7 @@
     <t>products/trucks/series/hx</t>
   </si>
   <si>
-    <t>2026-10-18T02:35:47.987Z</t>
+    <t>2026-10-18T06:29:06.470Z</t>
   </si>
   <si>
     <t>HX® Series | International®</t>
@@ -3607,7 +3607,7 @@
     <t>products/trucks/series/lt</t>
   </si>
   <si>
-    <t>2026-10-18T02:11:42.507Z</t>
+    <t>2026-10-18T06:05:27.183Z</t>
   </si>
   <si>
     <t>LT® Series | International®</t>
@@ -3625,7 +3625,7 @@
     <t>products/trucks/series/mv</t>
   </si>
   <si>
-    <t>2026-10-18T02:35:56.990Z</t>
+    <t>2026-10-18T06:29:14.985Z</t>
   </si>
   <si>
     <t>MV™ Series | International®</t>
@@ -3643,7 +3643,7 @@
     <t>products/trucks/series/rh</t>
   </si>
   <si>
-    <t>2026-10-18T02:36:05.222Z</t>
+    <t>2026-10-18T06:29:21.792Z</t>
   </si>
   <si>
     <t>RH™ Series | International®</t>
@@ -3661,7 +3661,7 @@
     <t>dealer-network/recruitment/influence-winners/2024-technician-of-the-year/rookies</t>
   </si>
   <si>
-    <t>2026-10-18T02:12:44.212Z</t>
+    <t>2026-10-18T06:06:25.692Z</t>
   </si>
   <si>
     <t>Rookie Technicians of the Year | International®</t>
@@ -3676,7 +3676,7 @@
     <t>dealer-network/recruitment/influence-winners/2024-technician-of-the-year/veterans</t>
   </si>
   <si>
-    <t>2026-10-18T02:12:51.672Z</t>
+    <t>2026-10-18T06:06:34.154Z</t>
   </si>
   <si>
     <t>Veteran Technicians of the Year | International®</t>
@@ -3691,7 +3691,7 @@
     <t>fr/products/trucks/classes/heavy</t>
   </si>
   <si>
-    <t>2026-10-18T02:13:25.392Z</t>
+    <t>2026-10-18T06:07:10.157Z</t>
   </si>
   <si>
     <t>Camions Poids Lourd | International®</t>
@@ -3706,7 +3706,7 @@
     <t>fr/products/trucks/classes/medium</t>
   </si>
   <si>
-    <t>2026-10-18T02:13:31.816Z</t>
+    <t>2026-10-18T06:07:17.851Z</t>
   </si>
   <si>
     <t>Camions de Poids Moyen | International®</t>
@@ -3721,7 +3721,7 @@
     <t>fr/products/trucks/classes/severe</t>
   </si>
   <si>
-    <t>2026-10-18T02:13:37.675Z</t>
+    <t>2026-10-18T06:07:24.698Z</t>
   </si>
   <si>
     <t>Camions de Service Intense | International®</t>
@@ -3739,7 +3739,7 @@
     <t>fr/products/trucks/series/cv</t>
   </si>
   <si>
-    <t>2026-10-18T02:13:45.768Z</t>
+    <t>2026-10-18T06:07:31.670Z</t>
   </si>
   <si>
     <t>Série CV | International®</t>
@@ -3757,7 +3757,7 @@
     <t>fr/products/trucks/series/electric-mv</t>
   </si>
   <si>
-    <t>2026-10-18T02:13:52.997Z</t>
+    <t>2026-10-18T06:07:39.200Z</t>
   </si>
   <si>
     <t>Série eMV | International®</t>
@@ -3775,7 +3775,7 @@
     <t>fr/products/trucks/series/hv</t>
   </si>
   <si>
-    <t>2026-10-18T02:13:59.028Z</t>
+    <t>2026-10-18T06:07:45.769Z</t>
   </si>
   <si>
     <t>Série HV | International®</t>
@@ -3793,7 +3793,7 @@
     <t>fr/products/trucks/series/hx</t>
   </si>
   <si>
-    <t>2026-10-18T02:14:05.049Z</t>
+    <t>2026-10-18T06:07:52.219Z</t>
   </si>
   <si>
     <t>Série HX | International®</t>
@@ -3811,7 +3811,7 @@
     <t>fr/products/trucks/series/lt</t>
   </si>
   <si>
-    <t>2026-10-18T02:14:11.839Z</t>
+    <t>2026-10-18T06:07:59.013Z</t>
   </si>
   <si>
     <t>Série LT | International®</t>
@@ -3829,7 +3829,7 @@
     <t>fr/products/trucks/series/mv</t>
   </si>
   <si>
-    <t>2026-10-18T02:14:20.112Z</t>
+    <t>2026-10-18T06:08:06.620Z</t>
   </si>
   <si>
     <t>Série MV | International®</t>
@@ -3847,7 +3847,7 @@
     <t>fr/products/trucks/series/rh</t>
   </si>
   <si>
-    <t>2026-10-18T02:14:28.182Z</t>
+    <t>2026-10-18T06:08:13.667Z</t>
   </si>
   <si>
     <t>Série RH | International®</t>
@@ -3865,7 +3865,7 @@
     <t>products/trucks/features/engines-and-powertrains/battery-electric-powertrains</t>
   </si>
   <si>
-    <t>2026-10-18T02:34:33.739Z</t>
+    <t>2026-10-18T06:27:47.824Z</t>
   </si>
   <si>
     <t>Battery Electric Powertrains | International®</t>
@@ -3883,7 +3883,7 @@
     <t>products/trucks/features/engines-and-powertrains/cummins-b6-7</t>
   </si>
   <si>
-    <t>2026-10-18T02:34:41.539Z</t>
+    <t>2026-10-18T06:27:55.374Z</t>
   </si>
   <si>
     <t>Cummins® B6.7 | International®</t>
@@ -3901,7 +3901,7 @@
     <t>products/trucks/features/engines-and-powertrains/cummins-l9</t>
   </si>
   <si>
-    <t>2026-10-18T02:34:47.894Z</t>
+    <t>2026-10-18T06:28:03.433Z</t>
   </si>
   <si>
     <t>Cummins® L9 | International®</t>
@@ -3919,7 +3919,7 @@
     <t>products/trucks/features/engines-and-powertrains/cummins-x15</t>
   </si>
   <si>
-    <t>2026-10-18T02:34:54.157Z</t>
+    <t>2026-10-18T06:28:10.491Z</t>
   </si>
   <si>
     <t>Cummins® X15 | International®</t>

</xml_diff>